<commit_message>
feat: formalizar dirección regional y avance dinámico
</commit_message>
<xml_diff>
--- a/cms/Sistema_Evidencias_OPS_CMS.xlsx
+++ b/cms/Sistema_Evidencias_OPS_CMS.xlsx
@@ -2109,11 +2109,6 @@
           <t>CMS · Gerentes de Distrito</t>
         </is>
       </c>
-      <c r="B1" s="14" t="n"/>
-      <c r="C1" s="14" t="n"/>
-      <c r="D1" s="14" t="n"/>
-      <c r="E1" s="14" t="n"/>
-      <c r="F1" s="14" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
@@ -2122,7 +2117,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -3107,12 +3101,6 @@
           <t>CMS · Organigrama Región | Centro's</t>
         </is>
       </c>
-      <c r="B1" s="14" t="n"/>
-      <c r="C1" s="14" t="n"/>
-      <c r="D1" s="14" t="n"/>
-      <c r="E1" s="14" t="n"/>
-      <c r="F1" s="14" t="n"/>
-      <c r="G1" s="14" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="20" t="inlineStr">
@@ -3169,7 +3157,7 @@
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Raúl Sierra</t>
+          <t>Raúl Sinohe Sierra Santa Maria</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -3348,10 +3336,6 @@
           <t>CMS · Tiendas Abiertas</t>
         </is>
       </c>
-      <c r="B1" s="14" t="n"/>
-      <c r="C1" s="14" t="n"/>
-      <c r="D1" s="14" t="n"/>
-      <c r="E1" s="14" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="18" t="inlineStr">
@@ -13064,7 +13048,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Formalizar dirección regional y avance dinámico (#6)
CMS, Python, Hero, navegación y porcentajes regionales auditados.
</commit_message>
<xml_diff>
--- a/cms/Sistema_Evidencias_OPS_CMS.xlsx
+++ b/cms/Sistema_Evidencias_OPS_CMS.xlsx
@@ -2109,11 +2109,6 @@
           <t>CMS · Gerentes de Distrito</t>
         </is>
       </c>
-      <c r="B1" s="14" t="n"/>
-      <c r="C1" s="14" t="n"/>
-      <c r="D1" s="14" t="n"/>
-      <c r="E1" s="14" t="n"/>
-      <c r="F1" s="14" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
@@ -2122,7 +2117,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -3107,12 +3101,6 @@
           <t>CMS · Organigrama Región | Centro's</t>
         </is>
       </c>
-      <c r="B1" s="14" t="n"/>
-      <c r="C1" s="14" t="n"/>
-      <c r="D1" s="14" t="n"/>
-      <c r="E1" s="14" t="n"/>
-      <c r="F1" s="14" t="n"/>
-      <c r="G1" s="14" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="20" t="inlineStr">
@@ -3169,7 +3157,7 @@
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Raúl Sierra</t>
+          <t>Raúl Sinohe Sierra Santa Maria</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -3348,10 +3336,6 @@
           <t>CMS · Tiendas Abiertas</t>
         </is>
       </c>
-      <c r="B1" s="14" t="n"/>
-      <c r="C1" s="14" t="n"/>
-      <c r="D1" s="14" t="n"/>
-      <c r="E1" s="14" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="18" t="inlineStr">
@@ -13064,7 +13048,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: estabilizar lectura CeCo y CeCo1
</commit_message>
<xml_diff>
--- a/cms/Sistema_Evidencias_OPS_CMS.xlsx
+++ b/cms/Sistema_Evidencias_OPS_CMS.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actividades" sheetId="1" r:id="Rd69528b13f0345a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gerentes" sheetId="2" r:id="R4db4c06ffd8f4693"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Organigrama" sheetId="3" r:id="R6e800e54c4db4aff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiendas Abiertas" sheetId="4" r:id="Rfa197e560a5e4679"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuracion" sheetId="5" r:id="Re4ae619cd6a945cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actividades" sheetId="1" r:id="R0573a88a9a2a4493"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gerentes" sheetId="2" r:id="R7abd3811458a4709"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Organigrama" sheetId="3" r:id="R05be1645096345a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiendas Abiertas" sheetId="4" r:id="Rcd17933bbb8b4bb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuracion" sheetId="5" r:id="R0a11951dfa5844ee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2077,7 +2077,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1af1cb86d0b4ae2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80e3dfc694354c53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3097,7 +3097,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcfd5e23ca7504bef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d16f6df4b974957"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13267,15 +13267,9 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
-      <x:c r="A16" s="23" t="str">
-        <x:v>ignoredResponseIds</x:v>
-      </x:c>
-      <x:c r="B16" s="23" t="str">
-        <x:v>353</x:v>
-      </x:c>
-      <x:c r="C16" s="27" t="str">
-        <x:v>Ids originales de Forms excluidos temporalmente como pruebas; no bloquea respuestas reales del CeCo</x:v>
-      </x:c>
+      <x:c r="A16" s="23"/>
+      <x:c r="B16" s="23"/>
+      <x:c r="C16" s="27"/>
     </x:row>
     <x:row r="17" ht="8" customHeight="1"/>
   </x:sheetData>
@@ -13290,7 +13284,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fe6a9c4613247c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79b1cd2b8dbf4bbd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: estabilizar lectura CeCo y CeCo1 (#8)
</commit_message>
<xml_diff>
--- a/cms/Sistema_Evidencias_OPS_CMS.xlsx
+++ b/cms/Sistema_Evidencias_OPS_CMS.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actividades" sheetId="1" r:id="Rd69528b13f0345a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gerentes" sheetId="2" r:id="R4db4c06ffd8f4693"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Organigrama" sheetId="3" r:id="R6e800e54c4db4aff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiendas Abiertas" sheetId="4" r:id="Rfa197e560a5e4679"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuracion" sheetId="5" r:id="Re4ae619cd6a945cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actividades" sheetId="1" r:id="R0573a88a9a2a4493"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gerentes" sheetId="2" r:id="R7abd3811458a4709"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Organigrama" sheetId="3" r:id="R05be1645096345a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiendas Abiertas" sheetId="4" r:id="Rcd17933bbb8b4bb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuracion" sheetId="5" r:id="R0a11951dfa5844ee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2077,7 +2077,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1af1cb86d0b4ae2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80e3dfc694354c53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3097,7 +3097,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcfd5e23ca7504bef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d16f6df4b974957"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13267,15 +13267,9 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
-      <x:c r="A16" s="23" t="str">
-        <x:v>ignoredResponseIds</x:v>
-      </x:c>
-      <x:c r="B16" s="23" t="str">
-        <x:v>353</x:v>
-      </x:c>
-      <x:c r="C16" s="27" t="str">
-        <x:v>Ids originales de Forms excluidos temporalmente como pruebas; no bloquea respuestas reales del CeCo</x:v>
-      </x:c>
+      <x:c r="A16" s="23"/>
+      <x:c r="B16" s="23"/>
+      <x:c r="C16" s="27"/>
     </x:row>
     <x:row r="17" ht="8" customHeight="1"/>
   </x:sheetData>
@@ -13290,7 +13284,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fe6a9c4613247c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79b1cd2b8dbf4bbd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>